<commit_message>
Cambios minimos en Excel
</commit_message>
<xml_diff>
--- a/SmartFactory VLSM.xlsx
+++ b/SmartFactory VLSM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Delta\Desktop\Cisco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23B6E28-1A20-465B-A3FD-1A431B6CB390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1762D992-2B42-4245-AF1A-7B25A8D52B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11460" yWindow="2940" windowWidth="13725" windowHeight="11835" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7455" yWindow="1860" windowWidth="13725" windowHeight="11835" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabla VLSM" sheetId="1" r:id="rId1"/>
@@ -781,9 +781,6 @@
     <t>Laptop-PT (Cliente VPN)</t>
   </si>
   <si>
-    <t>NO conectado (cliente VPN externo)</t>
-  </si>
-  <si>
     <t>NO (nube Internet simulada)</t>
   </si>
   <si>
@@ -803,6 +800,9 @@
   </si>
   <si>
     <t>Telefono-IoT</t>
+  </si>
+  <si>
+    <t>Conectado (Simulacion de Cliente VPN)</t>
   </si>
 </sst>
 </file>
@@ -2553,10 +2553,10 @@
     </row>
     <row r="12" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>254</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>185</v>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>202</v>
@@ -2926,7 +2926,7 @@
         <v>123</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>167</v>
@@ -3109,7 +3109,7 @@
         <v>166</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D42" s="19" t="s">
         <v>218</v>
@@ -3316,7 +3316,7 @@
         <v>218</v>
       </c>
       <c r="B53" s="30" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C53" s="30" t="s">
         <v>237</v>
@@ -3426,19 +3426,19 @@
         <v>249</v>
       </c>
       <c r="B59" s="30" t="s">
-        <v>202</v>
+        <v>166</v>
       </c>
       <c r="C59" s="30" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="D59" s="31" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="E59" s="30" t="s">
         <v>139</v>
       </c>
       <c r="F59" s="31" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -3458,7 +3458,7 @@
         <v>139</v>
       </c>
       <c r="F60" s="31" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>